<commit_message>
added descriptions to metrics
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics.xlsx
+++ b/wr_sdm/documentation/objectives_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{FD1E08C4-6B27-4B45-8835-65FC3284CB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51196FFB-E9B5-476D-9147-0F89637441DB}"/>
+  <xr:revisionPtr revIDLastSave="158" documentId="8_{FD1E08C4-6B27-4B45-8835-65FC3284CB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EB3A874-9963-405D-8E2E-B8B650DDC8C6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="67">
   <si>
     <t>objective</t>
   </si>
@@ -157,42 +157,9 @@
     <t>objective_description</t>
   </si>
   <si>
-    <t>Represents an interest in increasing salmonid abundance across the CV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Represents an interest in having growing or stable salmonid populations. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Represents an interest in increasing and maintaining the distribution of salmonids across historically occupied watersheds. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Estimated with models as annual number of hatchery returning adult spawning salmonids in each tributary, tracked each year of the 20-year simulation. Hatchery adult returns for each year and tributary are calculated by subtracting natural returning spawners from total spawners. Model results are summarized to show average Central Valley annual hatchery spawners. </t>
   </si>
   <si>
-    <t>Represents an interest in preserving life history diversity and fitness in natural populations.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Represents an interest in preserving life history diversity and fitness in natural populations. </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Salmonid models can be used to estimate the variation in juvenile abundance of each life stage (fry, parr, yearling) and calculate variation across years. Size distribution of juveniles is summarized in a single metric by using a Shannon diversity index. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Natural-origin juveniles are apportioned based on the annual proportion of natural fish based on hatchery releases</t>
-    </r>
-  </si>
-  <si>
-    <t>Salmonid models can be used to estimate the variation in juvenile abundance by month. Timing of juveniles at ocean entry is summarized in a single metric by using a Shannon diversity index. Timing varies by month. Natural-origin juveniles are apportioned based on the annual proportion of natural fish based on hatchery releases</t>
-  </si>
-  <si>
     <t xml:space="preserve">Estimated as number of years spawners decrease in abundance. Values are summarized across years and watersheds. </t>
   </si>
   <si>
@@ -206,21 +173,6 @@
   </si>
   <si>
     <t>Mean natural smolts at ocean entry</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Estimated with models as the number of natural juveniles reaching Chipps Island. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Natural-origin juveniles are apportioned based on the annual proportion of natural fish based on hatchery releases</t>
-    </r>
   </si>
   <si>
     <r>
@@ -245,22 +197,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">. Model results are summarized to show average Central Valley annual natural-origin spawners. </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">CRR can be estimated with models as the adult natural origin return ratio in each tributary, tracked for 20 years. CRR is calculated as the number of natural origin adult returns in year X+3 divided by the number of in-river spawners in year X. CRR is calculated for each year and tributary and then </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1C1D1F"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>averaged across years by watershed.</t>
     </r>
   </si>
   <si>
@@ -290,8 +226,68 @@
     </r>
   </si>
   <si>
+    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met all thresholds thresholds for the last 3 years of the dataset that have data, this was considered an independent population. Historic habitats include the Pit River, McCloud River, and Little Sacramento River.</t>
+  </si>
+  <si>
+    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met the thresholds for the last 3 years of the dataset that have data, this was considered an independent population.</t>
+  </si>
+  <si>
+    <t>Populations that have WRCS but do not meet all of the criteria for an independent population were considered dependent populations.</t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">Spawner outputs are filtered to include only tributary spawners. Model results are summarized to show average annual spawners </t>
+      <t xml:space="preserve">Estimated with models as the number of natural juveniles reaching Chipps Island. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Natural-origin juveniles are apportioned based on the annual proportion of natural fish based on hatchery releases</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Values are summarized to show average annual smolts at ocean entry. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Juvenile outputs are filtered to include only tributary juveniles. Results are summarized to show average annual juveniles </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>across tributaries</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Spawner outputs are filtered to include only tributary spawners. Results are summarized to show average annual spawners </t>
     </r>
     <r>
       <rPr>
@@ -316,40 +312,48 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Salmonid models can be used to estimate the annual variation of size (small, medium, large, very large) in juveniles at ocean entry. Size distribution of juveniles is summarized in a single metric by using a Shannon diversity index. Model results are summarized to show average annual diversity across tributaries. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Represents an interest in preserving life history diversity and fitness in WRCS populations. </t>
+  </si>
+  <si>
+    <t>Represents an interest in preserving life history diversity and fitness in WRCS populations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Represents an interest in having growing or stable WRCS populations. </t>
+  </si>
+  <si>
+    <t>Represents an interest in increasing WRCS abundance across the CV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Represents an interest in increasing and maintaining the distribution of WRCS across historically occupied watersheds. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salmonid models can be used to estimate the annual variation of outmigration timing (as measured by month) in natural-origin juveniles at ocean entry. Timing of juveniles at ocean entry is summarized in a single metric by using a Shannon diversity index. Model results are summarized to show average annual diversity across tributaries. </t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">Juvenile outputs are filtered to include only tributary juveniles. Model results are summarized to show average annual juveniles </t>
+      <t xml:space="preserve">CRR can be estimated with models as the adult natural origin return ratio in each tributary, tracked for 20 years. CRR is calculated as the number of natural origin adult returns in year X+3 divided by the number of total spawners in year X. CRR is calculated for each year and tributary and then </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF1C1D1F"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>across tributaries</t>
+      <t>averaged across years by watershed.</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met the thresholds for the last 3 years of the dataset with data, this was considered an independent population.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -495,6 +499,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF1C1D1F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -862,7 +872,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1285,7 +1295,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>42</v>
@@ -1305,10 +1315,10 @@
         <v>9</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1325,10 +1335,10 @@
         <v>11</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -1345,10 +1355,10 @@
         <v>13</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1362,13 +1372,13 @@
         <v>14</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1385,13 +1395,13 @@
         <v>18</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
@@ -1402,13 +1412,13 @@
         <v>19</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1425,10 +1435,10 @@
         <v>21</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1445,10 +1455,10 @@
         <v>25</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1465,10 +1475,10 @@
         <v>27</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1485,10 +1495,10 @@
         <v>29</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1505,10 +1515,10 @@
         <v>33</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1525,13 +1535,13 @@
         <v>35</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:6" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
@@ -1545,10 +1555,10 @@
         <v>37</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
@@ -1565,10 +1575,10 @@
         <v>39</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1585,9 +1595,11 @@
         <v>41</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17" s="5"/>
+        <v>64</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>55</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
edits the objectives_metrics.xlsx to address bolded and red text
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics.xlsx
+++ b/wr_sdm/documentation/objectives_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liz/Documents/code/winterRunSDM/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="158" documentId="8_{FD1E08C4-6B27-4B45-8835-65FC3284CB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EB3A874-9963-405D-8E2E-B8B650DDC8C6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA2B084-451A-B846-B1C3-832B03BEEC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
+    <workbookView xWindow="-37300" yWindow="-720" windowWidth="34800" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
   <sheets>
     <sheet name="objectives_metrics" sheetId="1" r:id="rId1"/>
@@ -175,18 +175,43 @@
     <t>Mean natural smolts at ocean entry</t>
   </si>
   <si>
+    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met the thresholds for the last 3 years of the dataset that have data, this was considered an independent population.</t>
+  </si>
+  <si>
+    <t>Populations that have WRCS but do not meet all of the criteria for an independent population were considered dependent populations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salmonid models can be used to estimate the annual variation of size (small, medium, large, very large) in juveniles at ocean entry. Size distribution of juveniles is summarized in a single metric by using a Shannon diversity index. Model results are summarized to show average annual diversity across tributaries. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Represents an interest in preserving life history diversity and fitness in WRCS populations. </t>
+  </si>
+  <si>
+    <t>Represents an interest in preserving life history diversity and fitness in WRCS populations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Represents an interest in having growing or stable WRCS populations. </t>
+  </si>
+  <si>
+    <t>Represents an interest in increasing WRCS abundance across the CV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Represents an interest in increasing and maintaining the distribution of WRCS across historically occupied watersheds. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salmonid models can be used to estimate the annual variation of outmigration timing (as measured by month) in natural-origin juveniles at ocean entry. Timing of juveniles at ocean entry is summarized in a single metric by using a Shannon diversity index. Model results are summarized to show average annual diversity across tributaries. </t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Estimated with models as annual number of natural returning adult spawning salmonids in each tributary, tracked each year of the 20-year simulation. Natural adult returns for each year and tributary are calculated by </t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>multiplying annual spawners by the annual  proportion of natural fish based on hatchery resleases</t>
+      <t>multiplying annual spawners by the annual  proportion of natural fish, calculated using juvenile hatchery proportions from previous years.</t>
     </r>
     <r>
       <rPr>
@@ -196,43 +221,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">. Model results are summarized to show average Central Valley annual natural-origin spawners. </t>
+      <t xml:space="preserve"> Model results are summarized to show average Central Valley annual natural-origin spawners. </t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Proportion of hatchery spawners can be estimated by multiplying the proportion of natural fish by the total spawners. Model results are summarized to show average annual pHOS </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1C1D1F"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>by watershed</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1C1D1F"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met all thresholds thresholds for the last 3 years of the dataset that have data, this was considered an independent population. Historic habitats include the Pit River, McCloud River, and Little Sacramento River.</t>
-  </si>
-  <si>
-    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met the thresholds for the last 3 years of the dataset that have data, this was considered an independent population.</t>
-  </si>
-  <si>
-    <t>Populations that have WRCS but do not meet all of the criteria for an independent population were considered dependent populations.</t>
   </si>
   <si>
     <r>
@@ -241,12 +231,10 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>Natural-origin juveniles are apportioned based on the annual proportion of natural fish based on hatchery releases</t>
+      <t>Natural-origin juveniles are calculated by applying the proportion of hatchery juveniles from the beginning of the simulation year</t>
     </r>
     <r>
       <rPr>
@@ -261,76 +249,48 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Juvenile outputs are filtered to include only tributary juveniles. Results are summarized to show average annual juveniles </t>
+      <t>Proportion of hatchery spawners is estimated by multiplying the proportion of natural adults by the total spawners. Model results are summarized to show average annual pHOS</t>
     </r>
     <r>
       <rPr>
-        <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF1C1D1F"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>across tributaries</t>
+      <t xml:space="preserve"> by watershed.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Spawner outputs are filtered to include only tributary spawners. Results are summarized to show average annual spawners </t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>.</t>
+      <t xml:space="preserve">across tributaries. </t>
     </r>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Spawner outputs are filtered to include only tributary spawners. Results are summarized to show average annual spawners </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>across tributaries</t>
+      <t xml:space="preserve">Juvenile outputs are filtered to include only tributary juveniles. Results are summarized to show average annual juveniles </t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">. </t>
+      <t>across tributaries.</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Salmonid models can be used to estimate the annual variation of size (small, medium, large, very large) in juveniles at ocean entry. Size distribution of juveniles is summarized in a single metric by using a Shannon diversity index. Model results are summarized to show average annual diversity across tributaries. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Represents an interest in preserving life history diversity and fitness in WRCS populations. </t>
-  </si>
-  <si>
-    <t>Represents an interest in preserving life history diversity and fitness in WRCS populations.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Represents an interest in having growing or stable WRCS populations. </t>
-  </si>
-  <si>
-    <t>Represents an interest in increasing WRCS abundance across the CV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Represents an interest in increasing and maintaining the distribution of WRCS across historically occupied watersheds. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salmonid models can be used to estimate the annual variation of outmigration timing (as measured by month) in natural-origin juveniles at ocean entry. Timing of juveniles at ocean entry is summarized in a single metric by using a Shannon diversity index. Model results are summarized to show average annual diversity across tributaries. </t>
+    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met all thresholds thresholds for the last 3 years of the dataset that have data, this was considered an independent population. Historic habitats represented in this process are the Pit River, McCloud River, and Little Sacramento River.</t>
   </si>
   <si>
     <r>
@@ -338,11 +298,9 @@
     </r>
     <r>
       <rPr>
-        <b/>
         <sz val="11"/>
         <color rgb="FF1C1D1F"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>averaged across years by watershed.</t>
@@ -353,7 +311,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,17 +454,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF1C1D1F"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -851,7 +818,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -863,16 +830,13 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1251,17 +1215,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8836ECF4-9848-4446-86BB-5107A1A11EC0}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="73.7109375" customWidth="1"/>
+    <col min="3" max="3" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="73.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1281,324 +1245,324 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="2" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F3" s="6" t="s">
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="2" customFormat="1" ht="96" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="2" customFormat="1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" s="7" t="s">
+    <row r="17" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="2" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>